<commit_message>
✨ feat(floxml): add transient solve settings support
- Add overall_transient (start_time, end_time, duration, keypoint_tolerance)
- Add time_patches with step control and distribution settings
- Add save_times for solution snapshot points
- Auto-set <modeling>/<transient>true when transient config is present
- Update example JSON and Excel template with transient sheets

Generated with [Claude Code](https://claude.ai/code)
via [Happy](https://happy.engineering)

Co-Authored-By: Claude <noreply@anthropic.com>
Co-Authored-By: Happy <yesreply@happy.engineering>
</commit_message>
<xml_diff>
--- a/solve_settings.example.xlsx
+++ b/solve_settings.example.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="overall_control" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="variable_controls" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="solver_controls" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="transient_overall" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="transient_save_times" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="time_patches" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -791,4 +794,217 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>end_time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>keypoint_tolerance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>save_time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>end_time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>step_control</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>minimum_number</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>step_distribution</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>distribution_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>minimum_number</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>increasing_power</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>minimum_number</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>